<commit_message>
web scraping first level
</commit_message>
<xml_diff>
--- a/sales.xlsx
+++ b/sales.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yashraj\Personal\Learning\AI Artifical Intelligence\Sample GenaI Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gyash\GenAI_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597D83E1-7D47-41F4-BDEE-DF263599036F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDDE3B44-3BB7-44E1-AD2A-CA2EE4B12F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -114,9 +114,6 @@
     <t>Electronics</t>
   </si>
   <si>
-    <t>Furniture</t>
-  </si>
-  <si>
     <t>Home Décor</t>
   </si>
   <si>
@@ -178,6 +175,9 @@
   </si>
   <si>
     <t>Story book</t>
+  </si>
+  <si>
+    <t>Home Office</t>
   </si>
 </sst>
 </file>
@@ -549,7 +549,7 @@
         <v>27</v>
       </c>
       <c r="F2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G2" s="1">
         <v>45658</v>
@@ -572,10 +572,10 @@
         <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G3" s="1">
         <v>45899</v>
@@ -598,10 +598,10 @@
         <v>25</v>
       </c>
       <c r="E4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" t="s">
         <v>40</v>
-      </c>
-      <c r="F4" t="s">
-        <v>41</v>
       </c>
       <c r="G4" s="1">
         <v>45986</v>
@@ -624,10 +624,10 @@
         <v>25</v>
       </c>
       <c r="E5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" t="s">
         <v>42</v>
-      </c>
-      <c r="F5" t="s">
-        <v>43</v>
       </c>
       <c r="G5" s="1">
         <v>46022</v>
@@ -650,10 +650,10 @@
         <v>26</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G6" s="1">
         <v>46054</v>
@@ -676,10 +676,10 @@
         <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G7" s="1">
         <v>45920</v>
@@ -702,10 +702,10 @@
         <v>25</v>
       </c>
       <c r="E8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" t="s">
         <v>44</v>
-      </c>
-      <c r="F8" t="s">
-        <v>45</v>
       </c>
       <c r="G8" s="1">
         <v>45679</v>
@@ -728,10 +728,10 @@
         <v>25</v>
       </c>
       <c r="E9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" t="s">
         <v>46</v>
-      </c>
-      <c r="F9" t="s">
-        <v>47</v>
       </c>
       <c r="G9" s="1">
         <v>45736</v>
@@ -754,10 +754,10 @@
         <v>25</v>
       </c>
       <c r="E10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" t="s">
         <v>48</v>
-      </c>
-      <c r="F10" t="s">
-        <v>49</v>
       </c>
       <c r="G10" s="1">
         <v>46101</v>
@@ -780,10 +780,10 @@
         <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G11" s="1">
         <v>46057</v>
@@ -806,10 +806,10 @@
         <v>25</v>
       </c>
       <c r="E12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" t="s">
         <v>30</v>
-      </c>
-      <c r="F12" t="s">
-        <v>31</v>
       </c>
       <c r="G12" s="1">
         <v>46021</v>
@@ -832,10 +832,10 @@
         <v>26</v>
       </c>
       <c r="E13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" t="s">
         <v>35</v>
-      </c>
-      <c r="F13" t="s">
-        <v>36</v>
       </c>
       <c r="G13" s="1">
         <v>45327</v>

</xml_diff>

<commit_message>
3 types of data ingestions v3
</commit_message>
<xml_diff>
--- a/sales.xlsx
+++ b/sales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gyash\GenAI_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDDE3B44-3BB7-44E1-AD2A-CA2EE4B12F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26488ACD-971C-41CD-99FB-6DEFE57B60B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="51">
   <si>
     <t>Cust_Name</t>
   </si>
@@ -178,6 +178,9 @@
   </si>
   <si>
     <t>Home Office</t>
+  </si>
+  <si>
+    <t>iPhone</t>
   </si>
 </sst>
 </file>
@@ -496,7 +499,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.44140625" bestFit="1" customWidth="1"/>
@@ -844,6 +847,58 @@
         <v>300</v>
       </c>
     </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="1">
+        <v>45241</v>
+      </c>
+      <c r="H14">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="1">
+        <v>45637</v>
+      </c>
+      <c r="H15">
+        <v>90000</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H12" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>